<commit_message>
feat: migrate validation rules and expand editable validation flow
</commit_message>
<xml_diff>
--- a/config/income_profit_rulebook_skeleton.xlsx
+++ b/config/income_profit_rulebook_skeleton.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="income_grouping" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="income_tree" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="income_formulas" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contribution_policy" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1346,13 +1347,289 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gp_share_mode</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>impact_when_mixed_or_total_negative</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>当前代码口径选择: impact_always / algebraic_always / impact_when_mixed_or_total_negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>impact_ratio_label</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>毛利贡献（驱动占比）</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>驱动占比标签（绝对值口径）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>algebraic_ratio_label</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>毛利贡献（占总毛利比例）</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>代数占比标签</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>basis_impact_text</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>按绝对值口径</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>口径说明文本</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>basis_algebraic_text</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>按代数口径</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>口径说明文本</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>net_attr_enabled</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>净归因占比是否启用（规划项）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>net_attr_ratio_label</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>对全部分项业务毛利影响总量的占比</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>净归因口径标签（规划项）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>net_attr_formula</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>segment_gp/ABS(total_gp)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>净归因计算公式（规划项）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>strength_ratio_label</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>影响强度占比（按绝对值）</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>驱动强度标签（规划项）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>strength_formula</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ABS(segment_gp)/SUM(ABS(segment_gp))</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>驱动强度计算公式（规划项）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>zero_total_policy</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>strength_only</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>总毛利为0时仅展示驱动占比（规划项）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>display_dual_caliber</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>前端并行展示净归因+驱动占比（规划项）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1557,7 +1834,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Algebraic GP Contribution</t>
+          <t>毛利代数占比</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1595,7 +1872,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Impact Share of GP</t>
+          <t>毛利驱动占比</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1622,6 +1899,44 @@
         <v>2</v>
       </c>
       <c r="H7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gp_net_attribution</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>毛利净归因占比</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>segment.gross_profit</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>abs(total.gross_profit)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ratio_signed_to_abs_total</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1712,17 +2027,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>increase</t>
+          <t>增加</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>decrease</t>
+          <t>减少</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>保持稳定</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -1750,17 +2065,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>up</t>
+          <t>增加</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>down</t>
+          <t>减少</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>保持稳定</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1788,17 +2103,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>increase</t>
+          <t>增加</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>decrease</t>
+          <t>减少</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>保持稳定</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1826,17 +2141,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>up</t>
+          <t>增加</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>down</t>
+          <t>减少</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>保持稳定</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -1917,7 +2232,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>same-sign overall profit</t>
+          <t>总毛利为正-分项同号</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1932,16 +2247,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>profit contributor</t>
+          <t>利润贡献项</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>profit diluter</t>
+          <t>利润稀释项</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
@@ -1955,7 +2270,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>mixed-sign overall profit</t>
+          <t>总毛利为正-分项异号</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1970,16 +2285,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>profit contributor</t>
+          <t>利润贡献项</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>profit diluter</t>
+          <t>利润稀释项</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
@@ -1993,7 +2308,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>same-sign overall loss</t>
+          <t>总毛利为负-分项同号</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2008,16 +2323,16 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>loss offsetter</t>
+          <t>亏损抵减项</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>loss amplifier</t>
+          <t>亏损放大项</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -2031,7 +2346,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>mixed-sign overall loss</t>
+          <t>总毛利为负-分项异号</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2046,16 +2361,16 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>loss offsetter</t>
+          <t>亏损抵减项</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>loss amplifier</t>
+          <t>亏损放大项</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
@@ -2069,7 +2384,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>overall zero</t>
+          <t>总毛利为零-分项对冲</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2084,16 +2399,16 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>offset item</t>
+          <t>抵消项</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>drag item</t>
+          <t>拖累项</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
@@ -2335,7 +2650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2415,7 +2730,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>y1,r1,y2,r2,y3,r3,rt21,rt32</t>
+          <t>ratio_label,y1,r1,y2,r2,y3,r3,rt21,rt32</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -2460,15 +2775,290 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>毛利贡献（占总毛利比例）：{y1}年{i1}，{y2}年{i2}，{y3}年{i3}；{y2}较{y1}{it21}，{y3}较{y2}{it32}。</t>
+          <t>{ratio_label}：{y1}年{i1}，{y2}年{i2}，{y3}年{i3}；{y2}较{y1}{it21}，{y3}较{y2}{it32}。</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>y1,i1,y2,i2,y3,i3,it21,it32,direction</t>
+          <t>ratio_label,y1,i1,y2,i2,y3,i3,it21,it32</t>
         </is>
       </c>
       <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TPL_GP_BASIS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gross_contribution_basis</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>口径说明：{y1}年{b1}，{y2}年{b2}，{y3}年{b3}。</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>y1,b1,y2,b2,y3,b3</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TPL_GP_NET</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>gross_segment_net_attr</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>净归因占比：{y1}年{n1}，{y2}年{n2}，{y3}年{n3}；{y2}较{y1}{nt21}，{y3}较{y2}{nt32}。</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>y1,n1,y2,n2,y3,n3,nt21,nt32</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TPL_GP_DUAL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gross_segment_dual_view</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>{strength_label}：{s_latest}；{net_label}：{n_latest}。</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>strength_label,s_latest,net_label,n_latest</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TPL_GP_SCN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gross_segment_scenario_judgement</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>场景定性（{latest_year}）：{qual_word}（{scenario}）。</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>latest_year,qual_word,scenario</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TPL_PROF_HDR_MISS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>profit_summary_header_missing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>{title}?{latest_year}????????</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>title,latest_year</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TPL_PROF_HDR_POS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>profit_summary_header_positive</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>{title}?{latest_year}????{total_amount}???</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>title,latest_year,total_amount</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TPL_PROF_HDR_ZERO</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>profit_summary_header_zero</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>{title}?{latest_year}?????0??????????</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>title,latest_year</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TPL_PROF_HDR_NEG</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>profit_summary_header_negative</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>{title}?{latest_year}??????{total_abs_amount}???</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>title,latest_year,total_abs_amount</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TPL_PROF_LINE_POS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>profit_summary_line_positive</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>{name}???{amount}???{net_attr_label}{net_attr_pct}?{direction_word}?</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>name,amount,net_attr_label,net_attr_pct,direction_word</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TPL_PROF_LINE_NEG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>profit_summary_line_negative</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>{name}???{abs_amount}???{net_attr_label}{net_attr_pct}?{direction_word}?</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>name,abs_amount,net_attr_label,net_attr_pct,direction_word</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TPL_PROF_LINE_ZERO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>profit_summary_line_zero</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>{name}??????{net_attr_label}{net_attr_pct}?</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>name,net_attr_label,net_attr_pct</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>